<commit_message>
feat(camera): enhance Excel import utility and UI responsiveness
Add a string normalization method to improve header validation by removing special characters. Update the UI state management to handle submission flags during the import process, ensuring accurate feedback on import status and error handling.
</commit_message>
<xml_diff>
--- a/assets/Camera_Template_Import.xlsx
+++ b/assets/Camera_Template_Import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hieunt1/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B142B05-B24E-BA49-A1E8-AD7EA5935070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CECA0BA4-E7A4-CE47-B756-909AE8E28D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="620" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="40740" yWindow="1860" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang tính1" sheetId="1" r:id="rId1"/>
@@ -37,15 +37,11 @@
     <t>Password</t>
   </si>
   <si>
+    <t>Địa chỉ RTSP</t>
+  </si>
+  <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Địa chỉ ONVIF
+      <t xml:space="preserve">Địa chỉ ONVIF 
 </t>
     </r>
     <r>
@@ -60,17 +56,7 @@
     </r>
   </si>
   <si>
-    <t>Địa chỉ RTSP</t>
-  </si>
-  <si>
     <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">Địa chỉ luồng phụ 
 </t>
     </r>
@@ -169,7 +155,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -180,6 +166,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -403,15 +395,14 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="9.1640625" customWidth="1"/>
-    <col min="3" max="3" width="17.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" customWidth="1"/>
     <col min="6" max="6" width="40.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.83203125" customWidth="1"/>
+    <col min="7" max="8" width="44.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:30" ht="28" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -427,13 +418,13 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="7" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1"/>
@@ -458,6 +449,8 @@
       <c r="AD1" s="1"/>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A2" s="4"/>
+      <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -466,6 +459,8 @@
       <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
@@ -3462,11 +3457,6 @@
       <c r="G1000" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B3" xr:uid="{103C61E6-0E54-6540-A6EA-850BC28CDC93}">
-      <formula1>"ONVIF,RTSP"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: update Camera_Template_Import.xlsx file
</commit_message>
<xml_diff>
--- a/assets/Camera_Template_Import.xlsx
+++ b/assets/Camera_Template_Import.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hieunt1/Downloads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CECA0BA4-E7A4-CE47-B756-909AE8E28D21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864E1197-9ECB-4B48-92DD-E2758CBA7521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="40740" yWindow="1860" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="43080" yWindow="620" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Trang tính1" sheetId="1" r:id="rId1"/>
@@ -399,7 +399,8 @@
     <col min="4" max="4" width="9" customWidth="1"/>
     <col min="5" max="5" width="10.6640625" customWidth="1"/>
     <col min="6" max="6" width="40.33203125" bestFit="1" customWidth="1"/>
-    <col min="7" max="8" width="44.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="50.5" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:30" ht="28" x14ac:dyDescent="0.15">
@@ -450,7 +451,6 @@
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
       <c r="C2" s="4"/>
       <c r="D2" s="4"/>
       <c r="E2" s="4"/>
@@ -460,7 +460,6 @@
     </row>
     <row r="3" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="4"/>
-      <c r="B3" s="4"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
@@ -3457,6 +3456,11 @@
       <c r="G1000" s="3"/>
     </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B50" xr:uid="{B931C216-68A0-CE42-887D-3F465506B7E6}">
+      <formula1>"ONVIF,RTSP"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(export): update Excel export functionality and template handling
This commit enhances the export functionality by incorporating a template for Excel files, ensuring that headers are dynamically generated based on the template. It also updates the version of the 'meta' and 'test_api' packages in the pubspec.lock file, and modifies the Camera_Template_Import.xlsx file. Additionally, it refines the header validation process in the Excel utility to improve data integrity during imports.
</commit_message>
<xml_diff>
--- a/assets/Camera_Template_Import.xlsx
+++ b/assets/Camera_Template_Import.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hieunt1/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/hieuvivas/vms_flutter_client/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{864E1197-9ECB-4B48-92DD-E2758CBA7521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D286B2-2D29-5B42-8ACC-8F0973FF9C95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="620" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="620" windowWidth="33720" windowHeight="20980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Trang tính1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -128,18 +128,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor rgb="FFFFFF00"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -155,20 +149,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -407,7 +395,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -419,13 +407,13 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>7</v>
       </c>
       <c r="I1" s="1"/>
@@ -450,3010 +438,3010 @@
       <c r="AD1" s="1"/>
     </row>
     <row r="2" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A3" s="4"/>
-      <c r="C3" s="4"/>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="4"/>
+      <c r="A3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="3"/>
     </row>
     <row r="5" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G5" s="3"/>
+      <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G6" s="3"/>
+      <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G7" s="3"/>
+      <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G8" s="3"/>
+      <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G9" s="3"/>
+      <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G10" s="3"/>
+      <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G11" s="3"/>
+      <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G12" s="3"/>
+      <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G13" s="3"/>
+      <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G14" s="3"/>
+      <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G15" s="3"/>
+      <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:30" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G16" s="3"/>
+      <c r="G16" s="2"/>
     </row>
     <row r="17" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G17" s="3"/>
+      <c r="G17" s="2"/>
     </row>
     <row r="18" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G18" s="3"/>
+      <c r="G18" s="2"/>
     </row>
     <row r="19" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G19" s="3"/>
+      <c r="G19" s="2"/>
     </row>
     <row r="20" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G20" s="3"/>
+      <c r="G20" s="2"/>
     </row>
     <row r="21" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G21" s="3"/>
+      <c r="G21" s="2"/>
     </row>
     <row r="22" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G22" s="3"/>
+      <c r="G22" s="2"/>
     </row>
     <row r="23" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G23" s="3"/>
+      <c r="G23" s="2"/>
     </row>
     <row r="24" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G24" s="3"/>
+      <c r="G24" s="2"/>
     </row>
     <row r="25" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G25" s="3"/>
+      <c r="G25" s="2"/>
     </row>
     <row r="26" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G26" s="3"/>
+      <c r="G26" s="2"/>
     </row>
     <row r="27" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G27" s="3"/>
+      <c r="G27" s="2"/>
     </row>
     <row r="28" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G28" s="3"/>
+      <c r="G28" s="2"/>
     </row>
     <row r="29" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G29" s="3"/>
+      <c r="G29" s="2"/>
     </row>
     <row r="30" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G30" s="3"/>
+      <c r="G30" s="2"/>
     </row>
     <row r="31" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G31" s="3"/>
+      <c r="G31" s="2"/>
     </row>
     <row r="32" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G32" s="3"/>
+      <c r="G32" s="2"/>
     </row>
     <row r="33" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G33" s="3"/>
+      <c r="G33" s="2"/>
     </row>
     <row r="34" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G34" s="3"/>
+      <c r="G34" s="2"/>
     </row>
     <row r="35" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G35" s="3"/>
+      <c r="G35" s="2"/>
     </row>
     <row r="36" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G36" s="3"/>
+      <c r="G36" s="2"/>
     </row>
     <row r="37" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G37" s="3"/>
+      <c r="G37" s="2"/>
     </row>
     <row r="38" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G38" s="3"/>
+      <c r="G38" s="2"/>
     </row>
     <row r="39" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G39" s="3"/>
+      <c r="G39" s="2"/>
     </row>
     <row r="40" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G40" s="3"/>
+      <c r="G40" s="2"/>
     </row>
     <row r="41" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G41" s="3"/>
+      <c r="G41" s="2"/>
     </row>
     <row r="42" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G42" s="3"/>
+      <c r="G42" s="2"/>
     </row>
     <row r="43" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G43" s="3"/>
+      <c r="G43" s="2"/>
     </row>
     <row r="44" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G44" s="3"/>
+      <c r="G44" s="2"/>
     </row>
     <row r="45" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G45" s="3"/>
+      <c r="G45" s="2"/>
     </row>
     <row r="46" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G46" s="3"/>
+      <c r="G46" s="2"/>
     </row>
     <row r="47" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G47" s="3"/>
+      <c r="G47" s="2"/>
     </row>
     <row r="48" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G48" s="3"/>
+      <c r="G48" s="2"/>
     </row>
     <row r="49" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G49" s="3"/>
+      <c r="G49" s="2"/>
     </row>
     <row r="50" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G50" s="3"/>
+      <c r="G50" s="2"/>
     </row>
     <row r="51" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G51" s="3"/>
+      <c r="G51" s="2"/>
     </row>
     <row r="52" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G52" s="3"/>
+      <c r="G52" s="2"/>
     </row>
     <row r="53" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G53" s="3"/>
+      <c r="G53" s="2"/>
     </row>
     <row r="54" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G54" s="3"/>
+      <c r="G54" s="2"/>
     </row>
     <row r="55" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G55" s="3"/>
+      <c r="G55" s="2"/>
     </row>
     <row r="56" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G56" s="3"/>
+      <c r="G56" s="2"/>
     </row>
     <row r="57" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G57" s="3"/>
+      <c r="G57" s="2"/>
     </row>
     <row r="58" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G58" s="3"/>
+      <c r="G58" s="2"/>
     </row>
     <row r="59" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G59" s="3"/>
+      <c r="G59" s="2"/>
     </row>
     <row r="60" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G60" s="3"/>
+      <c r="G60" s="2"/>
     </row>
     <row r="61" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G61" s="3"/>
+      <c r="G61" s="2"/>
     </row>
     <row r="62" spans="7:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="G62" s="3"/>
+      <c r="G62" s="2"/>
     </row>
     <row r="63" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G63" s="3"/>
+      <c r="G63" s="2"/>
     </row>
     <row r="64" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G64" s="3"/>
+      <c r="G64" s="2"/>
     </row>
     <row r="65" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G65" s="3"/>
+      <c r="G65" s="2"/>
     </row>
     <row r="66" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G66" s="3"/>
+      <c r="G66" s="2"/>
     </row>
     <row r="67" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G67" s="3"/>
+      <c r="G67" s="2"/>
     </row>
     <row r="68" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G68" s="3"/>
+      <c r="G68" s="2"/>
     </row>
     <row r="69" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G69" s="3"/>
+      <c r="G69" s="2"/>
     </row>
     <row r="70" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G70" s="3"/>
+      <c r="G70" s="2"/>
     </row>
     <row r="71" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G71" s="3"/>
+      <c r="G71" s="2"/>
     </row>
     <row r="72" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G72" s="3"/>
+      <c r="G72" s="2"/>
     </row>
     <row r="73" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G73" s="3"/>
+      <c r="G73" s="2"/>
     </row>
     <row r="74" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G74" s="3"/>
+      <c r="G74" s="2"/>
     </row>
     <row r="75" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G75" s="3"/>
+      <c r="G75" s="2"/>
     </row>
     <row r="76" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G76" s="3"/>
+      <c r="G76" s="2"/>
     </row>
     <row r="77" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G77" s="3"/>
+      <c r="G77" s="2"/>
     </row>
     <row r="78" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G78" s="3"/>
+      <c r="G78" s="2"/>
     </row>
     <row r="79" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G79" s="3"/>
+      <c r="G79" s="2"/>
     </row>
     <row r="80" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G80" s="3"/>
+      <c r="G80" s="2"/>
     </row>
     <row r="81" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G81" s="3"/>
+      <c r="G81" s="2"/>
     </row>
     <row r="82" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G82" s="3"/>
+      <c r="G82" s="2"/>
     </row>
     <row r="83" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G83" s="3"/>
+      <c r="G83" s="2"/>
     </row>
     <row r="84" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G84" s="3"/>
+      <c r="G84" s="2"/>
     </row>
     <row r="85" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G85" s="3"/>
+      <c r="G85" s="2"/>
     </row>
     <row r="86" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G86" s="3"/>
+      <c r="G86" s="2"/>
     </row>
     <row r="87" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G87" s="3"/>
+      <c r="G87" s="2"/>
     </row>
     <row r="88" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G88" s="3"/>
+      <c r="G88" s="2"/>
     </row>
     <row r="89" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G89" s="3"/>
+      <c r="G89" s="2"/>
     </row>
     <row r="90" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G90" s="3"/>
+      <c r="G90" s="2"/>
     </row>
     <row r="91" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G91" s="3"/>
+      <c r="G91" s="2"/>
     </row>
     <row r="92" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G92" s="3"/>
+      <c r="G92" s="2"/>
     </row>
     <row r="93" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G93" s="3"/>
+      <c r="G93" s="2"/>
     </row>
     <row r="94" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G94" s="3"/>
+      <c r="G94" s="2"/>
     </row>
     <row r="95" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G95" s="3"/>
+      <c r="G95" s="2"/>
     </row>
     <row r="96" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G96" s="3"/>
+      <c r="G96" s="2"/>
     </row>
     <row r="97" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G97" s="3"/>
+      <c r="G97" s="2"/>
     </row>
     <row r="98" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G98" s="3"/>
+      <c r="G98" s="2"/>
     </row>
     <row r="99" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G99" s="3"/>
+      <c r="G99" s="2"/>
     </row>
     <row r="100" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G100" s="3"/>
+      <c r="G100" s="2"/>
     </row>
     <row r="101" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G101" s="3"/>
+      <c r="G101" s="2"/>
     </row>
     <row r="102" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G102" s="3"/>
+      <c r="G102" s="2"/>
     </row>
     <row r="103" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G103" s="3"/>
+      <c r="G103" s="2"/>
     </row>
     <row r="104" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G104" s="3"/>
+      <c r="G104" s="2"/>
     </row>
     <row r="105" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G105" s="3"/>
+      <c r="G105" s="2"/>
     </row>
     <row r="106" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G106" s="3"/>
+      <c r="G106" s="2"/>
     </row>
     <row r="107" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G107" s="3"/>
+      <c r="G107" s="2"/>
     </row>
     <row r="108" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G108" s="3"/>
+      <c r="G108" s="2"/>
     </row>
     <row r="109" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G109" s="3"/>
+      <c r="G109" s="2"/>
     </row>
     <row r="110" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G110" s="3"/>
+      <c r="G110" s="2"/>
     </row>
     <row r="111" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G111" s="3"/>
+      <c r="G111" s="2"/>
     </row>
     <row r="112" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G112" s="3"/>
+      <c r="G112" s="2"/>
     </row>
     <row r="113" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G113" s="3"/>
+      <c r="G113" s="2"/>
     </row>
     <row r="114" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G114" s="3"/>
+      <c r="G114" s="2"/>
     </row>
     <row r="115" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G115" s="3"/>
+      <c r="G115" s="2"/>
     </row>
     <row r="116" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G116" s="3"/>
+      <c r="G116" s="2"/>
     </row>
     <row r="117" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G117" s="3"/>
+      <c r="G117" s="2"/>
     </row>
     <row r="118" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G118" s="3"/>
+      <c r="G118" s="2"/>
     </row>
     <row r="119" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G119" s="3"/>
+      <c r="G119" s="2"/>
     </row>
     <row r="120" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G120" s="3"/>
+      <c r="G120" s="2"/>
     </row>
     <row r="121" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G121" s="3"/>
+      <c r="G121" s="2"/>
     </row>
     <row r="122" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G122" s="3"/>
+      <c r="G122" s="2"/>
     </row>
     <row r="123" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G123" s="3"/>
+      <c r="G123" s="2"/>
     </row>
     <row r="124" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G124" s="3"/>
+      <c r="G124" s="2"/>
     </row>
     <row r="125" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G125" s="3"/>
+      <c r="G125" s="2"/>
     </row>
     <row r="126" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G126" s="3"/>
+      <c r="G126" s="2"/>
     </row>
     <row r="127" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G127" s="3"/>
+      <c r="G127" s="2"/>
     </row>
     <row r="128" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G128" s="3"/>
+      <c r="G128" s="2"/>
     </row>
     <row r="129" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G129" s="3"/>
+      <c r="G129" s="2"/>
     </row>
     <row r="130" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G130" s="3"/>
+      <c r="G130" s="2"/>
     </row>
     <row r="131" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G131" s="3"/>
+      <c r="G131" s="2"/>
     </row>
     <row r="132" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G132" s="3"/>
+      <c r="G132" s="2"/>
     </row>
     <row r="133" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G133" s="3"/>
+      <c r="G133" s="2"/>
     </row>
     <row r="134" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G134" s="3"/>
+      <c r="G134" s="2"/>
     </row>
     <row r="135" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G135" s="3"/>
+      <c r="G135" s="2"/>
     </row>
     <row r="136" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G136" s="3"/>
+      <c r="G136" s="2"/>
     </row>
     <row r="137" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G137" s="3"/>
+      <c r="G137" s="2"/>
     </row>
     <row r="138" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G138" s="3"/>
+      <c r="G138" s="2"/>
     </row>
     <row r="139" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G139" s="3"/>
+      <c r="G139" s="2"/>
     </row>
     <row r="140" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G140" s="3"/>
+      <c r="G140" s="2"/>
     </row>
     <row r="141" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G141" s="3"/>
+      <c r="G141" s="2"/>
     </row>
     <row r="142" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G142" s="3"/>
+      <c r="G142" s="2"/>
     </row>
     <row r="143" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G143" s="3"/>
+      <c r="G143" s="2"/>
     </row>
     <row r="144" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G144" s="3"/>
+      <c r="G144" s="2"/>
     </row>
     <row r="145" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G145" s="3"/>
+      <c r="G145" s="2"/>
     </row>
     <row r="146" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G146" s="3"/>
+      <c r="G146" s="2"/>
     </row>
     <row r="147" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G147" s="3"/>
+      <c r="G147" s="2"/>
     </row>
     <row r="148" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G148" s="3"/>
+      <c r="G148" s="2"/>
     </row>
     <row r="149" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G149" s="3"/>
+      <c r="G149" s="2"/>
     </row>
     <row r="150" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G150" s="3"/>
+      <c r="G150" s="2"/>
     </row>
     <row r="151" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G151" s="3"/>
+      <c r="G151" s="2"/>
     </row>
     <row r="152" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G152" s="3"/>
+      <c r="G152" s="2"/>
     </row>
     <row r="153" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G153" s="3"/>
+      <c r="G153" s="2"/>
     </row>
     <row r="154" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G154" s="3"/>
+      <c r="G154" s="2"/>
     </row>
     <row r="155" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G155" s="3"/>
+      <c r="G155" s="2"/>
     </row>
     <row r="156" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G156" s="3"/>
+      <c r="G156" s="2"/>
     </row>
     <row r="157" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G157" s="3"/>
+      <c r="G157" s="2"/>
     </row>
     <row r="158" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G158" s="3"/>
+      <c r="G158" s="2"/>
     </row>
     <row r="159" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G159" s="3"/>
+      <c r="G159" s="2"/>
     </row>
     <row r="160" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G160" s="3"/>
+      <c r="G160" s="2"/>
     </row>
     <row r="161" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G161" s="3"/>
+      <c r="G161" s="2"/>
     </row>
     <row r="162" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G162" s="3"/>
+      <c r="G162" s="2"/>
     </row>
     <row r="163" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G163" s="3"/>
+      <c r="G163" s="2"/>
     </row>
     <row r="164" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G164" s="3"/>
+      <c r="G164" s="2"/>
     </row>
     <row r="165" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G165" s="3"/>
+      <c r="G165" s="2"/>
     </row>
     <row r="166" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G166" s="3"/>
+      <c r="G166" s="2"/>
     </row>
     <row r="167" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G167" s="3"/>
+      <c r="G167" s="2"/>
     </row>
     <row r="168" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G168" s="3"/>
+      <c r="G168" s="2"/>
     </row>
     <row r="169" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G169" s="3"/>
+      <c r="G169" s="2"/>
     </row>
     <row r="170" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G170" s="3"/>
+      <c r="G170" s="2"/>
     </row>
     <row r="171" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G171" s="3"/>
+      <c r="G171" s="2"/>
     </row>
     <row r="172" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G172" s="3"/>
+      <c r="G172" s="2"/>
     </row>
     <row r="173" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G173" s="3"/>
+      <c r="G173" s="2"/>
     </row>
     <row r="174" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G174" s="3"/>
+      <c r="G174" s="2"/>
     </row>
     <row r="175" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G175" s="3"/>
+      <c r="G175" s="2"/>
     </row>
     <row r="176" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G176" s="3"/>
+      <c r="G176" s="2"/>
     </row>
     <row r="177" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G177" s="3"/>
+      <c r="G177" s="2"/>
     </row>
     <row r="178" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G178" s="3"/>
+      <c r="G178" s="2"/>
     </row>
     <row r="179" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G179" s="3"/>
+      <c r="G179" s="2"/>
     </row>
     <row r="180" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G180" s="3"/>
+      <c r="G180" s="2"/>
     </row>
     <row r="181" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G181" s="3"/>
+      <c r="G181" s="2"/>
     </row>
     <row r="182" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G182" s="3"/>
+      <c r="G182" s="2"/>
     </row>
     <row r="183" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G183" s="3"/>
+      <c r="G183" s="2"/>
     </row>
     <row r="184" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G184" s="3"/>
+      <c r="G184" s="2"/>
     </row>
     <row r="185" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G185" s="3"/>
+      <c r="G185" s="2"/>
     </row>
     <row r="186" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G186" s="3"/>
+      <c r="G186" s="2"/>
     </row>
     <row r="187" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G187" s="3"/>
+      <c r="G187" s="2"/>
     </row>
     <row r="188" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G188" s="3"/>
+      <c r="G188" s="2"/>
     </row>
     <row r="189" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G189" s="3"/>
+      <c r="G189" s="2"/>
     </row>
     <row r="190" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G190" s="3"/>
+      <c r="G190" s="2"/>
     </row>
     <row r="191" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G191" s="3"/>
+      <c r="G191" s="2"/>
     </row>
     <row r="192" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G192" s="3"/>
+      <c r="G192" s="2"/>
     </row>
     <row r="193" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G193" s="3"/>
+      <c r="G193" s="2"/>
     </row>
     <row r="194" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G194" s="3"/>
+      <c r="G194" s="2"/>
     </row>
     <row r="195" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G195" s="3"/>
+      <c r="G195" s="2"/>
     </row>
     <row r="196" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G196" s="3"/>
+      <c r="G196" s="2"/>
     </row>
     <row r="197" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G197" s="3"/>
+      <c r="G197" s="2"/>
     </row>
     <row r="198" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G198" s="3"/>
+      <c r="G198" s="2"/>
     </row>
     <row r="199" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G199" s="3"/>
+      <c r="G199" s="2"/>
     </row>
     <row r="200" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G200" s="3"/>
+      <c r="G200" s="2"/>
     </row>
     <row r="201" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G201" s="3"/>
+      <c r="G201" s="2"/>
     </row>
     <row r="202" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G202" s="3"/>
+      <c r="G202" s="2"/>
     </row>
     <row r="203" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G203" s="3"/>
+      <c r="G203" s="2"/>
     </row>
     <row r="204" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G204" s="3"/>
+      <c r="G204" s="2"/>
     </row>
     <row r="205" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G205" s="3"/>
+      <c r="G205" s="2"/>
     </row>
     <row r="206" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G206" s="3"/>
+      <c r="G206" s="2"/>
     </row>
     <row r="207" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G207" s="3"/>
+      <c r="G207" s="2"/>
     </row>
     <row r="208" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G208" s="3"/>
+      <c r="G208" s="2"/>
     </row>
     <row r="209" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G209" s="3"/>
+      <c r="G209" s="2"/>
     </row>
     <row r="210" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G210" s="3"/>
+      <c r="G210" s="2"/>
     </row>
     <row r="211" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G211" s="3"/>
+      <c r="G211" s="2"/>
     </row>
     <row r="212" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G212" s="3"/>
+      <c r="G212" s="2"/>
     </row>
     <row r="213" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G213" s="3"/>
+      <c r="G213" s="2"/>
     </row>
     <row r="214" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G214" s="3"/>
+      <c r="G214" s="2"/>
     </row>
     <row r="215" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G215" s="3"/>
+      <c r="G215" s="2"/>
     </row>
     <row r="216" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G216" s="3"/>
+      <c r="G216" s="2"/>
     </row>
     <row r="217" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G217" s="3"/>
+      <c r="G217" s="2"/>
     </row>
     <row r="218" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G218" s="3"/>
+      <c r="G218" s="2"/>
     </row>
     <row r="219" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G219" s="3"/>
+      <c r="G219" s="2"/>
     </row>
     <row r="220" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G220" s="3"/>
+      <c r="G220" s="2"/>
     </row>
     <row r="221" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G221" s="3"/>
+      <c r="G221" s="2"/>
     </row>
     <row r="222" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G222" s="3"/>
+      <c r="G222" s="2"/>
     </row>
     <row r="223" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G223" s="3"/>
+      <c r="G223" s="2"/>
     </row>
     <row r="224" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G224" s="3"/>
+      <c r="G224" s="2"/>
     </row>
     <row r="225" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G225" s="3"/>
+      <c r="G225" s="2"/>
     </row>
     <row r="226" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G226" s="3"/>
+      <c r="G226" s="2"/>
     </row>
     <row r="227" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G227" s="3"/>
+      <c r="G227" s="2"/>
     </row>
     <row r="228" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G228" s="3"/>
+      <c r="G228" s="2"/>
     </row>
     <row r="229" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G229" s="3"/>
+      <c r="G229" s="2"/>
     </row>
     <row r="230" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G230" s="3"/>
+      <c r="G230" s="2"/>
     </row>
     <row r="231" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G231" s="3"/>
+      <c r="G231" s="2"/>
     </row>
     <row r="232" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G232" s="3"/>
+      <c r="G232" s="2"/>
     </row>
     <row r="233" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G233" s="3"/>
+      <c r="G233" s="2"/>
     </row>
     <row r="234" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G234" s="3"/>
+      <c r="G234" s="2"/>
     </row>
     <row r="235" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G235" s="3"/>
+      <c r="G235" s="2"/>
     </row>
     <row r="236" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G236" s="3"/>
+      <c r="G236" s="2"/>
     </row>
     <row r="237" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G237" s="3"/>
+      <c r="G237" s="2"/>
     </row>
     <row r="238" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G238" s="3"/>
+      <c r="G238" s="2"/>
     </row>
     <row r="239" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G239" s="3"/>
+      <c r="G239" s="2"/>
     </row>
     <row r="240" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G240" s="3"/>
+      <c r="G240" s="2"/>
     </row>
     <row r="241" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G241" s="3"/>
+      <c r="G241" s="2"/>
     </row>
     <row r="242" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G242" s="3"/>
+      <c r="G242" s="2"/>
     </row>
     <row r="243" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G243" s="3"/>
+      <c r="G243" s="2"/>
     </row>
     <row r="244" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G244" s="3"/>
+      <c r="G244" s="2"/>
     </row>
     <row r="245" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G245" s="3"/>
+      <c r="G245" s="2"/>
     </row>
     <row r="246" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G246" s="3"/>
+      <c r="G246" s="2"/>
     </row>
     <row r="247" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G247" s="3"/>
+      <c r="G247" s="2"/>
     </row>
     <row r="248" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G248" s="3"/>
+      <c r="G248" s="2"/>
     </row>
     <row r="249" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G249" s="3"/>
+      <c r="G249" s="2"/>
     </row>
     <row r="250" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G250" s="3"/>
+      <c r="G250" s="2"/>
     </row>
     <row r="251" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G251" s="3"/>
+      <c r="G251" s="2"/>
     </row>
     <row r="252" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G252" s="3"/>
+      <c r="G252" s="2"/>
     </row>
     <row r="253" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G253" s="3"/>
+      <c r="G253" s="2"/>
     </row>
     <row r="254" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G254" s="3"/>
+      <c r="G254" s="2"/>
     </row>
     <row r="255" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G255" s="3"/>
+      <c r="G255" s="2"/>
     </row>
     <row r="256" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G256" s="3"/>
+      <c r="G256" s="2"/>
     </row>
     <row r="257" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G257" s="3"/>
+      <c r="G257" s="2"/>
     </row>
     <row r="258" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G258" s="3"/>
+      <c r="G258" s="2"/>
     </row>
     <row r="259" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G259" s="3"/>
+      <c r="G259" s="2"/>
     </row>
     <row r="260" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G260" s="3"/>
+      <c r="G260" s="2"/>
     </row>
     <row r="261" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G261" s="3"/>
+      <c r="G261" s="2"/>
     </row>
     <row r="262" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G262" s="3"/>
+      <c r="G262" s="2"/>
     </row>
     <row r="263" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G263" s="3"/>
+      <c r="G263" s="2"/>
     </row>
     <row r="264" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G264" s="3"/>
+      <c r="G264" s="2"/>
     </row>
     <row r="265" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G265" s="3"/>
+      <c r="G265" s="2"/>
     </row>
     <row r="266" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G266" s="3"/>
+      <c r="G266" s="2"/>
     </row>
     <row r="267" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G267" s="3"/>
+      <c r="G267" s="2"/>
     </row>
     <row r="268" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G268" s="3"/>
+      <c r="G268" s="2"/>
     </row>
     <row r="269" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G269" s="3"/>
+      <c r="G269" s="2"/>
     </row>
     <row r="270" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G270" s="3"/>
+      <c r="G270" s="2"/>
     </row>
     <row r="271" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G271" s="3"/>
+      <c r="G271" s="2"/>
     </row>
     <row r="272" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G272" s="3"/>
+      <c r="G272" s="2"/>
     </row>
     <row r="273" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G273" s="3"/>
+      <c r="G273" s="2"/>
     </row>
     <row r="274" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G274" s="3"/>
+      <c r="G274" s="2"/>
     </row>
     <row r="275" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G275" s="3"/>
+      <c r="G275" s="2"/>
     </row>
     <row r="276" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G276" s="3"/>
+      <c r="G276" s="2"/>
     </row>
     <row r="277" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G277" s="3"/>
+      <c r="G277" s="2"/>
     </row>
     <row r="278" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G278" s="3"/>
+      <c r="G278" s="2"/>
     </row>
     <row r="279" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G279" s="3"/>
+      <c r="G279" s="2"/>
     </row>
     <row r="280" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G280" s="3"/>
+      <c r="G280" s="2"/>
     </row>
     <row r="281" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G281" s="3"/>
+      <c r="G281" s="2"/>
     </row>
     <row r="282" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G282" s="3"/>
+      <c r="G282" s="2"/>
     </row>
     <row r="283" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G283" s="3"/>
+      <c r="G283" s="2"/>
     </row>
     <row r="284" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G284" s="3"/>
+      <c r="G284" s="2"/>
     </row>
     <row r="285" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G285" s="3"/>
+      <c r="G285" s="2"/>
     </row>
     <row r="286" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G286" s="3"/>
+      <c r="G286" s="2"/>
     </row>
     <row r="287" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G287" s="3"/>
+      <c r="G287" s="2"/>
     </row>
     <row r="288" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G288" s="3"/>
+      <c r="G288" s="2"/>
     </row>
     <row r="289" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G289" s="3"/>
+      <c r="G289" s="2"/>
     </row>
     <row r="290" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G290" s="3"/>
+      <c r="G290" s="2"/>
     </row>
     <row r="291" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G291" s="3"/>
+      <c r="G291" s="2"/>
     </row>
     <row r="292" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G292" s="3"/>
+      <c r="G292" s="2"/>
     </row>
     <row r="293" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G293" s="3"/>
+      <c r="G293" s="2"/>
     </row>
     <row r="294" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G294" s="3"/>
+      <c r="G294" s="2"/>
     </row>
     <row r="295" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G295" s="3"/>
+      <c r="G295" s="2"/>
     </row>
     <row r="296" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G296" s="3"/>
+      <c r="G296" s="2"/>
     </row>
     <row r="297" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G297" s="3"/>
+      <c r="G297" s="2"/>
     </row>
     <row r="298" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G298" s="3"/>
+      <c r="G298" s="2"/>
     </row>
     <row r="299" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G299" s="3"/>
+      <c r="G299" s="2"/>
     </row>
     <row r="300" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G300" s="3"/>
+      <c r="G300" s="2"/>
     </row>
     <row r="301" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G301" s="3"/>
+      <c r="G301" s="2"/>
     </row>
     <row r="302" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G302" s="3"/>
+      <c r="G302" s="2"/>
     </row>
     <row r="303" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G303" s="3"/>
+      <c r="G303" s="2"/>
     </row>
     <row r="304" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G304" s="3"/>
+      <c r="G304" s="2"/>
     </row>
     <row r="305" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G305" s="3"/>
+      <c r="G305" s="2"/>
     </row>
     <row r="306" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G306" s="3"/>
+      <c r="G306" s="2"/>
     </row>
     <row r="307" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G307" s="3"/>
+      <c r="G307" s="2"/>
     </row>
     <row r="308" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G308" s="3"/>
+      <c r="G308" s="2"/>
     </row>
     <row r="309" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G309" s="3"/>
+      <c r="G309" s="2"/>
     </row>
     <row r="310" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G310" s="3"/>
+      <c r="G310" s="2"/>
     </row>
     <row r="311" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G311" s="3"/>
+      <c r="G311" s="2"/>
     </row>
     <row r="312" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G312" s="3"/>
+      <c r="G312" s="2"/>
     </row>
     <row r="313" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G313" s="3"/>
+      <c r="G313" s="2"/>
     </row>
     <row r="314" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G314" s="3"/>
+      <c r="G314" s="2"/>
     </row>
     <row r="315" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G315" s="3"/>
+      <c r="G315" s="2"/>
     </row>
     <row r="316" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G316" s="3"/>
+      <c r="G316" s="2"/>
     </row>
     <row r="317" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G317" s="3"/>
+      <c r="G317" s="2"/>
     </row>
     <row r="318" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G318" s="3"/>
+      <c r="G318" s="2"/>
     </row>
     <row r="319" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G319" s="3"/>
+      <c r="G319" s="2"/>
     </row>
     <row r="320" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G320" s="3"/>
+      <c r="G320" s="2"/>
     </row>
     <row r="321" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G321" s="3"/>
+      <c r="G321" s="2"/>
     </row>
     <row r="322" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G322" s="3"/>
+      <c r="G322" s="2"/>
     </row>
     <row r="323" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G323" s="3"/>
+      <c r="G323" s="2"/>
     </row>
     <row r="324" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G324" s="3"/>
+      <c r="G324" s="2"/>
     </row>
     <row r="325" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G325" s="3"/>
+      <c r="G325" s="2"/>
     </row>
     <row r="326" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G326" s="3"/>
+      <c r="G326" s="2"/>
     </row>
     <row r="327" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G327" s="3"/>
+      <c r="G327" s="2"/>
     </row>
     <row r="328" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G328" s="3"/>
+      <c r="G328" s="2"/>
     </row>
     <row r="329" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G329" s="3"/>
+      <c r="G329" s="2"/>
     </row>
     <row r="330" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G330" s="3"/>
+      <c r="G330" s="2"/>
     </row>
     <row r="331" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G331" s="3"/>
+      <c r="G331" s="2"/>
     </row>
     <row r="332" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G332" s="3"/>
+      <c r="G332" s="2"/>
     </row>
     <row r="333" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G333" s="3"/>
+      <c r="G333" s="2"/>
     </row>
     <row r="334" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G334" s="3"/>
+      <c r="G334" s="2"/>
     </row>
     <row r="335" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G335" s="3"/>
+      <c r="G335" s="2"/>
     </row>
     <row r="336" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G336" s="3"/>
+      <c r="G336" s="2"/>
     </row>
     <row r="337" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G337" s="3"/>
+      <c r="G337" s="2"/>
     </row>
     <row r="338" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G338" s="3"/>
+      <c r="G338" s="2"/>
     </row>
     <row r="339" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G339" s="3"/>
+      <c r="G339" s="2"/>
     </row>
     <row r="340" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G340" s="3"/>
+      <c r="G340" s="2"/>
     </row>
     <row r="341" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G341" s="3"/>
+      <c r="G341" s="2"/>
     </row>
     <row r="342" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G342" s="3"/>
+      <c r="G342" s="2"/>
     </row>
     <row r="343" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G343" s="3"/>
+      <c r="G343" s="2"/>
     </row>
     <row r="344" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G344" s="3"/>
+      <c r="G344" s="2"/>
     </row>
     <row r="345" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G345" s="3"/>
+      <c r="G345" s="2"/>
     </row>
     <row r="346" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G346" s="3"/>
+      <c r="G346" s="2"/>
     </row>
     <row r="347" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G347" s="3"/>
+      <c r="G347" s="2"/>
     </row>
     <row r="348" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G348" s="3"/>
+      <c r="G348" s="2"/>
     </row>
     <row r="349" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G349" s="3"/>
+      <c r="G349" s="2"/>
     </row>
     <row r="350" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G350" s="3"/>
+      <c r="G350" s="2"/>
     </row>
     <row r="351" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G351" s="3"/>
+      <c r="G351" s="2"/>
     </row>
     <row r="352" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G352" s="3"/>
+      <c r="G352" s="2"/>
     </row>
     <row r="353" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G353" s="3"/>
+      <c r="G353" s="2"/>
     </row>
     <row r="354" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G354" s="3"/>
+      <c r="G354" s="2"/>
     </row>
     <row r="355" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G355" s="3"/>
+      <c r="G355" s="2"/>
     </row>
     <row r="356" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G356" s="3"/>
+      <c r="G356" s="2"/>
     </row>
     <row r="357" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G357" s="3"/>
+      <c r="G357" s="2"/>
     </row>
     <row r="358" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G358" s="3"/>
+      <c r="G358" s="2"/>
     </row>
     <row r="359" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G359" s="3"/>
+      <c r="G359" s="2"/>
     </row>
     <row r="360" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G360" s="3"/>
+      <c r="G360" s="2"/>
     </row>
     <row r="361" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G361" s="3"/>
+      <c r="G361" s="2"/>
     </row>
     <row r="362" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G362" s="3"/>
+      <c r="G362" s="2"/>
     </row>
     <row r="363" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G363" s="3"/>
+      <c r="G363" s="2"/>
     </row>
     <row r="364" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G364" s="3"/>
+      <c r="G364" s="2"/>
     </row>
     <row r="365" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G365" s="3"/>
+      <c r="G365" s="2"/>
     </row>
     <row r="366" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G366" s="3"/>
+      <c r="G366" s="2"/>
     </row>
     <row r="367" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G367" s="3"/>
+      <c r="G367" s="2"/>
     </row>
     <row r="368" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G368" s="3"/>
+      <c r="G368" s="2"/>
     </row>
     <row r="369" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G369" s="3"/>
+      <c r="G369" s="2"/>
     </row>
     <row r="370" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G370" s="3"/>
+      <c r="G370" s="2"/>
     </row>
     <row r="371" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G371" s="3"/>
+      <c r="G371" s="2"/>
     </row>
     <row r="372" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G372" s="3"/>
+      <c r="G372" s="2"/>
     </row>
     <row r="373" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G373" s="3"/>
+      <c r="G373" s="2"/>
     </row>
     <row r="374" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G374" s="3"/>
+      <c r="G374" s="2"/>
     </row>
     <row r="375" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G375" s="3"/>
+      <c r="G375" s="2"/>
     </row>
     <row r="376" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G376" s="3"/>
+      <c r="G376" s="2"/>
     </row>
     <row r="377" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G377" s="3"/>
+      <c r="G377" s="2"/>
     </row>
     <row r="378" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G378" s="3"/>
+      <c r="G378" s="2"/>
     </row>
     <row r="379" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G379" s="3"/>
+      <c r="G379" s="2"/>
     </row>
     <row r="380" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G380" s="3"/>
+      <c r="G380" s="2"/>
     </row>
     <row r="381" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G381" s="3"/>
+      <c r="G381" s="2"/>
     </row>
     <row r="382" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G382" s="3"/>
+      <c r="G382" s="2"/>
     </row>
     <row r="383" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G383" s="3"/>
+      <c r="G383" s="2"/>
     </row>
     <row r="384" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G384" s="3"/>
+      <c r="G384" s="2"/>
     </row>
     <row r="385" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G385" s="3"/>
+      <c r="G385" s="2"/>
     </row>
     <row r="386" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G386" s="3"/>
+      <c r="G386" s="2"/>
     </row>
     <row r="387" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G387" s="3"/>
+      <c r="G387" s="2"/>
     </row>
     <row r="388" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G388" s="3"/>
+      <c r="G388" s="2"/>
     </row>
     <row r="389" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G389" s="3"/>
+      <c r="G389" s="2"/>
     </row>
     <row r="390" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G390" s="3"/>
+      <c r="G390" s="2"/>
     </row>
     <row r="391" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G391" s="3"/>
+      <c r="G391" s="2"/>
     </row>
     <row r="392" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G392" s="3"/>
+      <c r="G392" s="2"/>
     </row>
     <row r="393" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G393" s="3"/>
+      <c r="G393" s="2"/>
     </row>
     <row r="394" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G394" s="3"/>
+      <c r="G394" s="2"/>
     </row>
     <row r="395" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G395" s="3"/>
+      <c r="G395" s="2"/>
     </row>
     <row r="396" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G396" s="3"/>
+      <c r="G396" s="2"/>
     </row>
     <row r="397" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G397" s="3"/>
+      <c r="G397" s="2"/>
     </row>
     <row r="398" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G398" s="3"/>
+      <c r="G398" s="2"/>
     </row>
     <row r="399" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G399" s="3"/>
+      <c r="G399" s="2"/>
     </row>
     <row r="400" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G400" s="3"/>
+      <c r="G400" s="2"/>
     </row>
     <row r="401" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G401" s="3"/>
+      <c r="G401" s="2"/>
     </row>
     <row r="402" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G402" s="3"/>
+      <c r="G402" s="2"/>
     </row>
     <row r="403" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G403" s="3"/>
+      <c r="G403" s="2"/>
     </row>
     <row r="404" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G404" s="3"/>
+      <c r="G404" s="2"/>
     </row>
     <row r="405" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G405" s="3"/>
+      <c r="G405" s="2"/>
     </row>
     <row r="406" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G406" s="3"/>
+      <c r="G406" s="2"/>
     </row>
     <row r="407" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G407" s="3"/>
+      <c r="G407" s="2"/>
     </row>
     <row r="408" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G408" s="3"/>
+      <c r="G408" s="2"/>
     </row>
     <row r="409" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G409" s="3"/>
+      <c r="G409" s="2"/>
     </row>
     <row r="410" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G410" s="3"/>
+      <c r="G410" s="2"/>
     </row>
     <row r="411" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G411" s="3"/>
+      <c r="G411" s="2"/>
     </row>
     <row r="412" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G412" s="3"/>
+      <c r="G412" s="2"/>
     </row>
     <row r="413" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G413" s="3"/>
+      <c r="G413" s="2"/>
     </row>
     <row r="414" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G414" s="3"/>
+      <c r="G414" s="2"/>
     </row>
     <row r="415" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G415" s="3"/>
+      <c r="G415" s="2"/>
     </row>
     <row r="416" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G416" s="3"/>
+      <c r="G416" s="2"/>
     </row>
     <row r="417" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G417" s="3"/>
+      <c r="G417" s="2"/>
     </row>
     <row r="418" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G418" s="3"/>
+      <c r="G418" s="2"/>
     </row>
     <row r="419" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G419" s="3"/>
+      <c r="G419" s="2"/>
     </row>
     <row r="420" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G420" s="3"/>
+      <c r="G420" s="2"/>
     </row>
     <row r="421" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G421" s="3"/>
+      <c r="G421" s="2"/>
     </row>
     <row r="422" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G422" s="3"/>
+      <c r="G422" s="2"/>
     </row>
     <row r="423" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G423" s="3"/>
+      <c r="G423" s="2"/>
     </row>
     <row r="424" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G424" s="3"/>
+      <c r="G424" s="2"/>
     </row>
     <row r="425" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G425" s="3"/>
+      <c r="G425" s="2"/>
     </row>
     <row r="426" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G426" s="3"/>
+      <c r="G426" s="2"/>
     </row>
     <row r="427" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G427" s="3"/>
+      <c r="G427" s="2"/>
     </row>
     <row r="428" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G428" s="3"/>
+      <c r="G428" s="2"/>
     </row>
     <row r="429" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G429" s="3"/>
+      <c r="G429" s="2"/>
     </row>
     <row r="430" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G430" s="3"/>
+      <c r="G430" s="2"/>
     </row>
     <row r="431" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G431" s="3"/>
+      <c r="G431" s="2"/>
     </row>
     <row r="432" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G432" s="3"/>
+      <c r="G432" s="2"/>
     </row>
     <row r="433" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G433" s="3"/>
+      <c r="G433" s="2"/>
     </row>
     <row r="434" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G434" s="3"/>
+      <c r="G434" s="2"/>
     </row>
     <row r="435" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G435" s="3"/>
+      <c r="G435" s="2"/>
     </row>
     <row r="436" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G436" s="3"/>
+      <c r="G436" s="2"/>
     </row>
     <row r="437" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G437" s="3"/>
+      <c r="G437" s="2"/>
     </row>
     <row r="438" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G438" s="3"/>
+      <c r="G438" s="2"/>
     </row>
     <row r="439" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G439" s="3"/>
+      <c r="G439" s="2"/>
     </row>
     <row r="440" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G440" s="3"/>
+      <c r="G440" s="2"/>
     </row>
     <row r="441" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G441" s="3"/>
+      <c r="G441" s="2"/>
     </row>
     <row r="442" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G442" s="3"/>
+      <c r="G442" s="2"/>
     </row>
     <row r="443" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G443" s="3"/>
+      <c r="G443" s="2"/>
     </row>
     <row r="444" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G444" s="3"/>
+      <c r="G444" s="2"/>
     </row>
     <row r="445" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G445" s="3"/>
+      <c r="G445" s="2"/>
     </row>
     <row r="446" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G446" s="3"/>
+      <c r="G446" s="2"/>
     </row>
     <row r="447" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G447" s="3"/>
+      <c r="G447" s="2"/>
     </row>
     <row r="448" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G448" s="3"/>
+      <c r="G448" s="2"/>
     </row>
     <row r="449" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G449" s="3"/>
+      <c r="G449" s="2"/>
     </row>
     <row r="450" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G450" s="3"/>
+      <c r="G450" s="2"/>
     </row>
     <row r="451" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G451" s="3"/>
+      <c r="G451" s="2"/>
     </row>
     <row r="452" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G452" s="3"/>
+      <c r="G452" s="2"/>
     </row>
     <row r="453" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G453" s="3"/>
+      <c r="G453" s="2"/>
     </row>
     <row r="454" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G454" s="3"/>
+      <c r="G454" s="2"/>
     </row>
     <row r="455" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G455" s="3"/>
+      <c r="G455" s="2"/>
     </row>
     <row r="456" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G456" s="3"/>
+      <c r="G456" s="2"/>
     </row>
     <row r="457" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G457" s="3"/>
+      <c r="G457" s="2"/>
     </row>
     <row r="458" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G458" s="3"/>
+      <c r="G458" s="2"/>
     </row>
     <row r="459" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G459" s="3"/>
+      <c r="G459" s="2"/>
     </row>
     <row r="460" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G460" s="3"/>
+      <c r="G460" s="2"/>
     </row>
     <row r="461" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G461" s="3"/>
+      <c r="G461" s="2"/>
     </row>
     <row r="462" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G462" s="3"/>
+      <c r="G462" s="2"/>
     </row>
     <row r="463" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G463" s="3"/>
+      <c r="G463" s="2"/>
     </row>
     <row r="464" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G464" s="3"/>
+      <c r="G464" s="2"/>
     </row>
     <row r="465" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G465" s="3"/>
+      <c r="G465" s="2"/>
     </row>
     <row r="466" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G466" s="3"/>
+      <c r="G466" s="2"/>
     </row>
     <row r="467" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G467" s="3"/>
+      <c r="G467" s="2"/>
     </row>
     <row r="468" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G468" s="3"/>
+      <c r="G468" s="2"/>
     </row>
     <row r="469" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G469" s="3"/>
+      <c r="G469" s="2"/>
     </row>
     <row r="470" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G470" s="3"/>
+      <c r="G470" s="2"/>
     </row>
     <row r="471" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G471" s="3"/>
+      <c r="G471" s="2"/>
     </row>
     <row r="472" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G472" s="3"/>
+      <c r="G472" s="2"/>
     </row>
     <row r="473" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G473" s="3"/>
+      <c r="G473" s="2"/>
     </row>
     <row r="474" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G474" s="3"/>
+      <c r="G474" s="2"/>
     </row>
     <row r="475" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G475" s="3"/>
+      <c r="G475" s="2"/>
     </row>
     <row r="476" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G476" s="3"/>
+      <c r="G476" s="2"/>
     </row>
     <row r="477" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G477" s="3"/>
+      <c r="G477" s="2"/>
     </row>
     <row r="478" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G478" s="3"/>
+      <c r="G478" s="2"/>
     </row>
     <row r="479" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G479" s="3"/>
+      <c r="G479" s="2"/>
     </row>
     <row r="480" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G480" s="3"/>
+      <c r="G480" s="2"/>
     </row>
     <row r="481" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G481" s="3"/>
+      <c r="G481" s="2"/>
     </row>
     <row r="482" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G482" s="3"/>
+      <c r="G482" s="2"/>
     </row>
     <row r="483" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G483" s="3"/>
+      <c r="G483" s="2"/>
     </row>
     <row r="484" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G484" s="3"/>
+      <c r="G484" s="2"/>
     </row>
     <row r="485" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G485" s="3"/>
+      <c r="G485" s="2"/>
     </row>
     <row r="486" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G486" s="3"/>
+      <c r="G486" s="2"/>
     </row>
     <row r="487" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G487" s="3"/>
+      <c r="G487" s="2"/>
     </row>
     <row r="488" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G488" s="3"/>
+      <c r="G488" s="2"/>
     </row>
     <row r="489" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G489" s="3"/>
+      <c r="G489" s="2"/>
     </row>
     <row r="490" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G490" s="3"/>
+      <c r="G490" s="2"/>
     </row>
     <row r="491" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G491" s="3"/>
+      <c r="G491" s="2"/>
     </row>
     <row r="492" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G492" s="3"/>
+      <c r="G492" s="2"/>
     </row>
     <row r="493" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G493" s="3"/>
+      <c r="G493" s="2"/>
     </row>
     <row r="494" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G494" s="3"/>
+      <c r="G494" s="2"/>
     </row>
     <row r="495" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G495" s="3"/>
+      <c r="G495" s="2"/>
     </row>
     <row r="496" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G496" s="3"/>
+      <c r="G496" s="2"/>
     </row>
     <row r="497" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G497" s="3"/>
+      <c r="G497" s="2"/>
     </row>
     <row r="498" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G498" s="3"/>
+      <c r="G498" s="2"/>
     </row>
     <row r="499" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G499" s="3"/>
+      <c r="G499" s="2"/>
     </row>
     <row r="500" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G500" s="3"/>
+      <c r="G500" s="2"/>
     </row>
     <row r="501" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G501" s="3"/>
+      <c r="G501" s="2"/>
     </row>
     <row r="502" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G502" s="3"/>
+      <c r="G502" s="2"/>
     </row>
     <row r="503" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G503" s="3"/>
+      <c r="G503" s="2"/>
     </row>
     <row r="504" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G504" s="3"/>
+      <c r="G504" s="2"/>
     </row>
     <row r="505" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G505" s="3"/>
+      <c r="G505" s="2"/>
     </row>
     <row r="506" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G506" s="3"/>
+      <c r="G506" s="2"/>
     </row>
     <row r="507" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G507" s="3"/>
+      <c r="G507" s="2"/>
     </row>
     <row r="508" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G508" s="3"/>
+      <c r="G508" s="2"/>
     </row>
     <row r="509" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G509" s="3"/>
+      <c r="G509" s="2"/>
     </row>
     <row r="510" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G510" s="3"/>
+      <c r="G510" s="2"/>
     </row>
     <row r="511" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G511" s="3"/>
+      <c r="G511" s="2"/>
     </row>
     <row r="512" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G512" s="3"/>
+      <c r="G512" s="2"/>
     </row>
     <row r="513" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G513" s="3"/>
+      <c r="G513" s="2"/>
     </row>
     <row r="514" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G514" s="3"/>
+      <c r="G514" s="2"/>
     </row>
     <row r="515" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G515" s="3"/>
+      <c r="G515" s="2"/>
     </row>
     <row r="516" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G516" s="3"/>
+      <c r="G516" s="2"/>
     </row>
     <row r="517" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G517" s="3"/>
+      <c r="G517" s="2"/>
     </row>
     <row r="518" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G518" s="3"/>
+      <c r="G518" s="2"/>
     </row>
     <row r="519" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G519" s="3"/>
+      <c r="G519" s="2"/>
     </row>
     <row r="520" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G520" s="3"/>
+      <c r="G520" s="2"/>
     </row>
     <row r="521" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G521" s="3"/>
+      <c r="G521" s="2"/>
     </row>
     <row r="522" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G522" s="3"/>
+      <c r="G522" s="2"/>
     </row>
     <row r="523" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G523" s="3"/>
+      <c r="G523" s="2"/>
     </row>
     <row r="524" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G524" s="3"/>
+      <c r="G524" s="2"/>
     </row>
     <row r="525" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G525" s="3"/>
+      <c r="G525" s="2"/>
     </row>
     <row r="526" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G526" s="3"/>
+      <c r="G526" s="2"/>
     </row>
     <row r="527" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G527" s="3"/>
+      <c r="G527" s="2"/>
     </row>
     <row r="528" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G528" s="3"/>
+      <c r="G528" s="2"/>
     </row>
     <row r="529" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G529" s="3"/>
+      <c r="G529" s="2"/>
     </row>
     <row r="530" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G530" s="3"/>
+      <c r="G530" s="2"/>
     </row>
     <row r="531" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G531" s="3"/>
+      <c r="G531" s="2"/>
     </row>
     <row r="532" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G532" s="3"/>
+      <c r="G532" s="2"/>
     </row>
     <row r="533" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G533" s="3"/>
+      <c r="G533" s="2"/>
     </row>
     <row r="534" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G534" s="3"/>
+      <c r="G534" s="2"/>
     </row>
     <row r="535" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G535" s="3"/>
+      <c r="G535" s="2"/>
     </row>
     <row r="536" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G536" s="3"/>
+      <c r="G536" s="2"/>
     </row>
     <row r="537" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G537" s="3"/>
+      <c r="G537" s="2"/>
     </row>
     <row r="538" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G538" s="3"/>
+      <c r="G538" s="2"/>
     </row>
     <row r="539" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G539" s="3"/>
+      <c r="G539" s="2"/>
     </row>
     <row r="540" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G540" s="3"/>
+      <c r="G540" s="2"/>
     </row>
     <row r="541" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G541" s="3"/>
+      <c r="G541" s="2"/>
     </row>
     <row r="542" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G542" s="3"/>
+      <c r="G542" s="2"/>
     </row>
     <row r="543" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G543" s="3"/>
+      <c r="G543" s="2"/>
     </row>
     <row r="544" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G544" s="3"/>
+      <c r="G544" s="2"/>
     </row>
     <row r="545" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G545" s="3"/>
+      <c r="G545" s="2"/>
     </row>
     <row r="546" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G546" s="3"/>
+      <c r="G546" s="2"/>
     </row>
     <row r="547" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G547" s="3"/>
+      <c r="G547" s="2"/>
     </row>
     <row r="548" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G548" s="3"/>
+      <c r="G548" s="2"/>
     </row>
     <row r="549" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G549" s="3"/>
+      <c r="G549" s="2"/>
     </row>
     <row r="550" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G550" s="3"/>
+      <c r="G550" s="2"/>
     </row>
     <row r="551" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G551" s="3"/>
+      <c r="G551" s="2"/>
     </row>
     <row r="552" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G552" s="3"/>
+      <c r="G552" s="2"/>
     </row>
     <row r="553" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G553" s="3"/>
+      <c r="G553" s="2"/>
     </row>
     <row r="554" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G554" s="3"/>
+      <c r="G554" s="2"/>
     </row>
     <row r="555" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G555" s="3"/>
+      <c r="G555" s="2"/>
     </row>
     <row r="556" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G556" s="3"/>
+      <c r="G556" s="2"/>
     </row>
     <row r="557" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G557" s="3"/>
+      <c r="G557" s="2"/>
     </row>
     <row r="558" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G558" s="3"/>
+      <c r="G558" s="2"/>
     </row>
     <row r="559" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G559" s="3"/>
+      <c r="G559" s="2"/>
     </row>
     <row r="560" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G560" s="3"/>
+      <c r="G560" s="2"/>
     </row>
     <row r="561" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G561" s="3"/>
+      <c r="G561" s="2"/>
     </row>
     <row r="562" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G562" s="3"/>
+      <c r="G562" s="2"/>
     </row>
     <row r="563" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G563" s="3"/>
+      <c r="G563" s="2"/>
     </row>
     <row r="564" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G564" s="3"/>
+      <c r="G564" s="2"/>
     </row>
     <row r="565" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G565" s="3"/>
+      <c r="G565" s="2"/>
     </row>
     <row r="566" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G566" s="3"/>
+      <c r="G566" s="2"/>
     </row>
     <row r="567" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G567" s="3"/>
+      <c r="G567" s="2"/>
     </row>
     <row r="568" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G568" s="3"/>
+      <c r="G568" s="2"/>
     </row>
     <row r="569" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G569" s="3"/>
+      <c r="G569" s="2"/>
     </row>
     <row r="570" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G570" s="3"/>
+      <c r="G570" s="2"/>
     </row>
     <row r="571" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G571" s="3"/>
+      <c r="G571" s="2"/>
     </row>
     <row r="572" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G572" s="3"/>
+      <c r="G572" s="2"/>
     </row>
     <row r="573" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G573" s="3"/>
+      <c r="G573" s="2"/>
     </row>
     <row r="574" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G574" s="3"/>
+      <c r="G574" s="2"/>
     </row>
     <row r="575" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G575" s="3"/>
+      <c r="G575" s="2"/>
     </row>
     <row r="576" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G576" s="3"/>
+      <c r="G576" s="2"/>
     </row>
     <row r="577" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G577" s="3"/>
+      <c r="G577" s="2"/>
     </row>
     <row r="578" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G578" s="3"/>
+      <c r="G578" s="2"/>
     </row>
     <row r="579" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G579" s="3"/>
+      <c r="G579" s="2"/>
     </row>
     <row r="580" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G580" s="3"/>
+      <c r="G580" s="2"/>
     </row>
     <row r="581" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G581" s="3"/>
+      <c r="G581" s="2"/>
     </row>
     <row r="582" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G582" s="3"/>
+      <c r="G582" s="2"/>
     </row>
     <row r="583" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G583" s="3"/>
+      <c r="G583" s="2"/>
     </row>
     <row r="584" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G584" s="3"/>
+      <c r="G584" s="2"/>
     </row>
     <row r="585" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G585" s="3"/>
+      <c r="G585" s="2"/>
     </row>
     <row r="586" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G586" s="3"/>
+      <c r="G586" s="2"/>
     </row>
     <row r="587" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G587" s="3"/>
+      <c r="G587" s="2"/>
     </row>
     <row r="588" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G588" s="3"/>
+      <c r="G588" s="2"/>
     </row>
     <row r="589" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G589" s="3"/>
+      <c r="G589" s="2"/>
     </row>
     <row r="590" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G590" s="3"/>
+      <c r="G590" s="2"/>
     </row>
     <row r="591" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G591" s="3"/>
+      <c r="G591" s="2"/>
     </row>
     <row r="592" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G592" s="3"/>
+      <c r="G592" s="2"/>
     </row>
     <row r="593" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G593" s="3"/>
+      <c r="G593" s="2"/>
     </row>
     <row r="594" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G594" s="3"/>
+      <c r="G594" s="2"/>
     </row>
     <row r="595" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G595" s="3"/>
+      <c r="G595" s="2"/>
     </row>
     <row r="596" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G596" s="3"/>
+      <c r="G596" s="2"/>
     </row>
     <row r="597" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G597" s="3"/>
+      <c r="G597" s="2"/>
     </row>
     <row r="598" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G598" s="3"/>
+      <c r="G598" s="2"/>
     </row>
     <row r="599" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G599" s="3"/>
+      <c r="G599" s="2"/>
     </row>
     <row r="600" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G600" s="3"/>
+      <c r="G600" s="2"/>
     </row>
     <row r="601" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G601" s="3"/>
+      <c r="G601" s="2"/>
     </row>
     <row r="602" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G602" s="3"/>
+      <c r="G602" s="2"/>
     </row>
     <row r="603" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G603" s="3"/>
+      <c r="G603" s="2"/>
     </row>
     <row r="604" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G604" s="3"/>
+      <c r="G604" s="2"/>
     </row>
     <row r="605" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G605" s="3"/>
+      <c r="G605" s="2"/>
     </row>
     <row r="606" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G606" s="3"/>
+      <c r="G606" s="2"/>
     </row>
     <row r="607" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G607" s="3"/>
+      <c r="G607" s="2"/>
     </row>
     <row r="608" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G608" s="3"/>
+      <c r="G608" s="2"/>
     </row>
     <row r="609" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G609" s="3"/>
+      <c r="G609" s="2"/>
     </row>
     <row r="610" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G610" s="3"/>
+      <c r="G610" s="2"/>
     </row>
     <row r="611" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G611" s="3"/>
+      <c r="G611" s="2"/>
     </row>
     <row r="612" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G612" s="3"/>
+      <c r="G612" s="2"/>
     </row>
     <row r="613" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G613" s="3"/>
+      <c r="G613" s="2"/>
     </row>
     <row r="614" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G614" s="3"/>
+      <c r="G614" s="2"/>
     </row>
     <row r="615" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G615" s="3"/>
+      <c r="G615" s="2"/>
     </row>
     <row r="616" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G616" s="3"/>
+      <c r="G616" s="2"/>
     </row>
     <row r="617" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G617" s="3"/>
+      <c r="G617" s="2"/>
     </row>
     <row r="618" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G618" s="3"/>
+      <c r="G618" s="2"/>
     </row>
     <row r="619" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G619" s="3"/>
+      <c r="G619" s="2"/>
     </row>
     <row r="620" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G620" s="3"/>
+      <c r="G620" s="2"/>
     </row>
     <row r="621" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G621" s="3"/>
+      <c r="G621" s="2"/>
     </row>
     <row r="622" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G622" s="3"/>
+      <c r="G622" s="2"/>
     </row>
     <row r="623" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G623" s="3"/>
+      <c r="G623" s="2"/>
     </row>
     <row r="624" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G624" s="3"/>
+      <c r="G624" s="2"/>
     </row>
     <row r="625" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G625" s="3"/>
+      <c r="G625" s="2"/>
     </row>
     <row r="626" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G626" s="3"/>
+      <c r="G626" s="2"/>
     </row>
     <row r="627" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G627" s="3"/>
+      <c r="G627" s="2"/>
     </row>
     <row r="628" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G628" s="3"/>
+      <c r="G628" s="2"/>
     </row>
     <row r="629" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G629" s="3"/>
+      <c r="G629" s="2"/>
     </row>
     <row r="630" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G630" s="3"/>
+      <c r="G630" s="2"/>
     </row>
     <row r="631" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G631" s="3"/>
+      <c r="G631" s="2"/>
     </row>
     <row r="632" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G632" s="3"/>
+      <c r="G632" s="2"/>
     </row>
     <row r="633" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G633" s="3"/>
+      <c r="G633" s="2"/>
     </row>
     <row r="634" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G634" s="3"/>
+      <c r="G634" s="2"/>
     </row>
     <row r="635" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G635" s="3"/>
+      <c r="G635" s="2"/>
     </row>
     <row r="636" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G636" s="3"/>
+      <c r="G636" s="2"/>
     </row>
     <row r="637" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G637" s="3"/>
+      <c r="G637" s="2"/>
     </row>
     <row r="638" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G638" s="3"/>
+      <c r="G638" s="2"/>
     </row>
     <row r="639" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G639" s="3"/>
+      <c r="G639" s="2"/>
     </row>
     <row r="640" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G640" s="3"/>
+      <c r="G640" s="2"/>
     </row>
     <row r="641" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G641" s="3"/>
+      <c r="G641" s="2"/>
     </row>
     <row r="642" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G642" s="3"/>
+      <c r="G642" s="2"/>
     </row>
     <row r="643" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G643" s="3"/>
+      <c r="G643" s="2"/>
     </row>
     <row r="644" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G644" s="3"/>
+      <c r="G644" s="2"/>
     </row>
     <row r="645" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G645" s="3"/>
+      <c r="G645" s="2"/>
     </row>
     <row r="646" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G646" s="3"/>
+      <c r="G646" s="2"/>
     </row>
     <row r="647" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G647" s="3"/>
+      <c r="G647" s="2"/>
     </row>
     <row r="648" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G648" s="3"/>
+      <c r="G648" s="2"/>
     </row>
     <row r="649" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G649" s="3"/>
+      <c r="G649" s="2"/>
     </row>
     <row r="650" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G650" s="3"/>
+      <c r="G650" s="2"/>
     </row>
     <row r="651" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G651" s="3"/>
+      <c r="G651" s="2"/>
     </row>
     <row r="652" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G652" s="3"/>
+      <c r="G652" s="2"/>
     </row>
     <row r="653" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G653" s="3"/>
+      <c r="G653" s="2"/>
     </row>
     <row r="654" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G654" s="3"/>
+      <c r="G654" s="2"/>
     </row>
     <row r="655" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G655" s="3"/>
+      <c r="G655" s="2"/>
     </row>
     <row r="656" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G656" s="3"/>
+      <c r="G656" s="2"/>
     </row>
     <row r="657" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G657" s="3"/>
+      <c r="G657" s="2"/>
     </row>
     <row r="658" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G658" s="3"/>
+      <c r="G658" s="2"/>
     </row>
     <row r="659" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G659" s="3"/>
+      <c r="G659" s="2"/>
     </row>
     <row r="660" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G660" s="3"/>
+      <c r="G660" s="2"/>
     </row>
     <row r="661" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G661" s="3"/>
+      <c r="G661" s="2"/>
     </row>
     <row r="662" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G662" s="3"/>
+      <c r="G662" s="2"/>
     </row>
     <row r="663" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G663" s="3"/>
+      <c r="G663" s="2"/>
     </row>
     <row r="664" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G664" s="3"/>
+      <c r="G664" s="2"/>
     </row>
     <row r="665" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G665" s="3"/>
+      <c r="G665" s="2"/>
     </row>
     <row r="666" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G666" s="3"/>
+      <c r="G666" s="2"/>
     </row>
     <row r="667" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G667" s="3"/>
+      <c r="G667" s="2"/>
     </row>
     <row r="668" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G668" s="3"/>
+      <c r="G668" s="2"/>
     </row>
     <row r="669" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G669" s="3"/>
+      <c r="G669" s="2"/>
     </row>
     <row r="670" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G670" s="3"/>
+      <c r="G670" s="2"/>
     </row>
     <row r="671" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G671" s="3"/>
+      <c r="G671" s="2"/>
     </row>
     <row r="672" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G672" s="3"/>
+      <c r="G672" s="2"/>
     </row>
     <row r="673" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G673" s="3"/>
+      <c r="G673" s="2"/>
     </row>
     <row r="674" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G674" s="3"/>
+      <c r="G674" s="2"/>
     </row>
     <row r="675" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G675" s="3"/>
+      <c r="G675" s="2"/>
     </row>
     <row r="676" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G676" s="3"/>
+      <c r="G676" s="2"/>
     </row>
     <row r="677" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G677" s="3"/>
+      <c r="G677" s="2"/>
     </row>
     <row r="678" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G678" s="3"/>
+      <c r="G678" s="2"/>
     </row>
     <row r="679" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G679" s="3"/>
+      <c r="G679" s="2"/>
     </row>
     <row r="680" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G680" s="3"/>
+      <c r="G680" s="2"/>
     </row>
     <row r="681" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G681" s="3"/>
+      <c r="G681" s="2"/>
     </row>
     <row r="682" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G682" s="3"/>
+      <c r="G682" s="2"/>
     </row>
     <row r="683" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G683" s="3"/>
+      <c r="G683" s="2"/>
     </row>
     <row r="684" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G684" s="3"/>
+      <c r="G684" s="2"/>
     </row>
     <row r="685" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G685" s="3"/>
+      <c r="G685" s="2"/>
     </row>
     <row r="686" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G686" s="3"/>
+      <c r="G686" s="2"/>
     </row>
     <row r="687" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G687" s="3"/>
+      <c r="G687" s="2"/>
     </row>
     <row r="688" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G688" s="3"/>
+      <c r="G688" s="2"/>
     </row>
     <row r="689" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G689" s="3"/>
+      <c r="G689" s="2"/>
     </row>
     <row r="690" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G690" s="3"/>
+      <c r="G690" s="2"/>
     </row>
     <row r="691" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G691" s="3"/>
+      <c r="G691" s="2"/>
     </row>
     <row r="692" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G692" s="3"/>
+      <c r="G692" s="2"/>
     </row>
     <row r="693" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G693" s="3"/>
+      <c r="G693" s="2"/>
     </row>
     <row r="694" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G694" s="3"/>
+      <c r="G694" s="2"/>
     </row>
     <row r="695" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G695" s="3"/>
+      <c r="G695" s="2"/>
     </row>
     <row r="696" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G696" s="3"/>
+      <c r="G696" s="2"/>
     </row>
     <row r="697" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G697" s="3"/>
+      <c r="G697" s="2"/>
     </row>
     <row r="698" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G698" s="3"/>
+      <c r="G698" s="2"/>
     </row>
     <row r="699" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G699" s="3"/>
+      <c r="G699" s="2"/>
     </row>
     <row r="700" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G700" s="3"/>
+      <c r="G700" s="2"/>
     </row>
     <row r="701" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G701" s="3"/>
+      <c r="G701" s="2"/>
     </row>
     <row r="702" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G702" s="3"/>
+      <c r="G702" s="2"/>
     </row>
     <row r="703" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G703" s="3"/>
+      <c r="G703" s="2"/>
     </row>
     <row r="704" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G704" s="3"/>
+      <c r="G704" s="2"/>
     </row>
     <row r="705" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G705" s="3"/>
+      <c r="G705" s="2"/>
     </row>
     <row r="706" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G706" s="3"/>
+      <c r="G706" s="2"/>
     </row>
     <row r="707" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G707" s="3"/>
+      <c r="G707" s="2"/>
     </row>
     <row r="708" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G708" s="3"/>
+      <c r="G708" s="2"/>
     </row>
     <row r="709" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G709" s="3"/>
+      <c r="G709" s="2"/>
     </row>
     <row r="710" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G710" s="3"/>
+      <c r="G710" s="2"/>
     </row>
     <row r="711" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G711" s="3"/>
+      <c r="G711" s="2"/>
     </row>
     <row r="712" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G712" s="3"/>
+      <c r="G712" s="2"/>
     </row>
     <row r="713" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G713" s="3"/>
+      <c r="G713" s="2"/>
     </row>
     <row r="714" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G714" s="3"/>
+      <c r="G714" s="2"/>
     </row>
     <row r="715" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G715" s="3"/>
+      <c r="G715" s="2"/>
     </row>
     <row r="716" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G716" s="3"/>
+      <c r="G716" s="2"/>
     </row>
     <row r="717" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G717" s="3"/>
+      <c r="G717" s="2"/>
     </row>
     <row r="718" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G718" s="3"/>
+      <c r="G718" s="2"/>
     </row>
     <row r="719" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G719" s="3"/>
+      <c r="G719" s="2"/>
     </row>
     <row r="720" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G720" s="3"/>
+      <c r="G720" s="2"/>
     </row>
     <row r="721" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G721" s="3"/>
+      <c r="G721" s="2"/>
     </row>
     <row r="722" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G722" s="3"/>
+      <c r="G722" s="2"/>
     </row>
     <row r="723" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G723" s="3"/>
+      <c r="G723" s="2"/>
     </row>
     <row r="724" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G724" s="3"/>
+      <c r="G724" s="2"/>
     </row>
     <row r="725" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G725" s="3"/>
+      <c r="G725" s="2"/>
     </row>
     <row r="726" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G726" s="3"/>
+      <c r="G726" s="2"/>
     </row>
     <row r="727" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G727" s="3"/>
+      <c r="G727" s="2"/>
     </row>
     <row r="728" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G728" s="3"/>
+      <c r="G728" s="2"/>
     </row>
     <row r="729" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G729" s="3"/>
+      <c r="G729" s="2"/>
     </row>
     <row r="730" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G730" s="3"/>
+      <c r="G730" s="2"/>
     </row>
     <row r="731" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G731" s="3"/>
+      <c r="G731" s="2"/>
     </row>
     <row r="732" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G732" s="3"/>
+      <c r="G732" s="2"/>
     </row>
     <row r="733" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G733" s="3"/>
+      <c r="G733" s="2"/>
     </row>
     <row r="734" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G734" s="3"/>
+      <c r="G734" s="2"/>
     </row>
     <row r="735" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G735" s="3"/>
+      <c r="G735" s="2"/>
     </row>
     <row r="736" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G736" s="3"/>
+      <c r="G736" s="2"/>
     </row>
     <row r="737" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G737" s="3"/>
+      <c r="G737" s="2"/>
     </row>
     <row r="738" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G738" s="3"/>
+      <c r="G738" s="2"/>
     </row>
     <row r="739" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G739" s="3"/>
+      <c r="G739" s="2"/>
     </row>
     <row r="740" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G740" s="3"/>
+      <c r="G740" s="2"/>
     </row>
     <row r="741" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G741" s="3"/>
+      <c r="G741" s="2"/>
     </row>
     <row r="742" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G742" s="3"/>
+      <c r="G742" s="2"/>
     </row>
     <row r="743" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G743" s="3"/>
+      <c r="G743" s="2"/>
     </row>
     <row r="744" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G744" s="3"/>
+      <c r="G744" s="2"/>
     </row>
     <row r="745" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G745" s="3"/>
+      <c r="G745" s="2"/>
     </row>
     <row r="746" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G746" s="3"/>
+      <c r="G746" s="2"/>
     </row>
     <row r="747" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G747" s="3"/>
+      <c r="G747" s="2"/>
     </row>
     <row r="748" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G748" s="3"/>
+      <c r="G748" s="2"/>
     </row>
     <row r="749" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G749" s="3"/>
+      <c r="G749" s="2"/>
     </row>
     <row r="750" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G750" s="3"/>
+      <c r="G750" s="2"/>
     </row>
     <row r="751" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G751" s="3"/>
+      <c r="G751" s="2"/>
     </row>
     <row r="752" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G752" s="3"/>
+      <c r="G752" s="2"/>
     </row>
     <row r="753" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G753" s="3"/>
+      <c r="G753" s="2"/>
     </row>
     <row r="754" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G754" s="3"/>
+      <c r="G754" s="2"/>
     </row>
     <row r="755" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G755" s="3"/>
+      <c r="G755" s="2"/>
     </row>
     <row r="756" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G756" s="3"/>
+      <c r="G756" s="2"/>
     </row>
     <row r="757" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G757" s="3"/>
+      <c r="G757" s="2"/>
     </row>
     <row r="758" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G758" s="3"/>
+      <c r="G758" s="2"/>
     </row>
     <row r="759" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G759" s="3"/>
+      <c r="G759" s="2"/>
     </row>
     <row r="760" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G760" s="3"/>
+      <c r="G760" s="2"/>
     </row>
     <row r="761" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G761" s="3"/>
+      <c r="G761" s="2"/>
     </row>
     <row r="762" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G762" s="3"/>
+      <c r="G762" s="2"/>
     </row>
     <row r="763" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G763" s="3"/>
+      <c r="G763" s="2"/>
     </row>
     <row r="764" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G764" s="3"/>
+      <c r="G764" s="2"/>
     </row>
     <row r="765" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G765" s="3"/>
+      <c r="G765" s="2"/>
     </row>
     <row r="766" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G766" s="3"/>
+      <c r="G766" s="2"/>
     </row>
     <row r="767" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G767" s="3"/>
+      <c r="G767" s="2"/>
     </row>
     <row r="768" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G768" s="3"/>
+      <c r="G768" s="2"/>
     </row>
     <row r="769" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G769" s="3"/>
+      <c r="G769" s="2"/>
     </row>
     <row r="770" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G770" s="3"/>
+      <c r="G770" s="2"/>
     </row>
     <row r="771" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G771" s="3"/>
+      <c r="G771" s="2"/>
     </row>
     <row r="772" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G772" s="3"/>
+      <c r="G772" s="2"/>
     </row>
     <row r="773" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G773" s="3"/>
+      <c r="G773" s="2"/>
     </row>
     <row r="774" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G774" s="3"/>
+      <c r="G774" s="2"/>
     </row>
     <row r="775" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G775" s="3"/>
+      <c r="G775" s="2"/>
     </row>
     <row r="776" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G776" s="3"/>
+      <c r="G776" s="2"/>
     </row>
     <row r="777" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G777" s="3"/>
+      <c r="G777" s="2"/>
     </row>
     <row r="778" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G778" s="3"/>
+      <c r="G778" s="2"/>
     </row>
     <row r="779" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G779" s="3"/>
+      <c r="G779" s="2"/>
     </row>
     <row r="780" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G780" s="3"/>
+      <c r="G780" s="2"/>
     </row>
     <row r="781" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G781" s="3"/>
+      <c r="G781" s="2"/>
     </row>
     <row r="782" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G782" s="3"/>
+      <c r="G782" s="2"/>
     </row>
     <row r="783" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G783" s="3"/>
+      <c r="G783" s="2"/>
     </row>
     <row r="784" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G784" s="3"/>
+      <c r="G784" s="2"/>
     </row>
     <row r="785" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G785" s="3"/>
+      <c r="G785" s="2"/>
     </row>
     <row r="786" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G786" s="3"/>
+      <c r="G786" s="2"/>
     </row>
     <row r="787" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G787" s="3"/>
+      <c r="G787" s="2"/>
     </row>
     <row r="788" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G788" s="3"/>
+      <c r="G788" s="2"/>
     </row>
     <row r="789" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G789" s="3"/>
+      <c r="G789" s="2"/>
     </row>
     <row r="790" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G790" s="3"/>
+      <c r="G790" s="2"/>
     </row>
     <row r="791" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G791" s="3"/>
+      <c r="G791" s="2"/>
     </row>
     <row r="792" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G792" s="3"/>
+      <c r="G792" s="2"/>
     </row>
     <row r="793" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G793" s="3"/>
+      <c r="G793" s="2"/>
     </row>
     <row r="794" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G794" s="3"/>
+      <c r="G794" s="2"/>
     </row>
     <row r="795" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G795" s="3"/>
+      <c r="G795" s="2"/>
     </row>
     <row r="796" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G796" s="3"/>
+      <c r="G796" s="2"/>
     </row>
     <row r="797" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G797" s="3"/>
+      <c r="G797" s="2"/>
     </row>
     <row r="798" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G798" s="3"/>
+      <c r="G798" s="2"/>
     </row>
     <row r="799" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G799" s="3"/>
+      <c r="G799" s="2"/>
     </row>
     <row r="800" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G800" s="3"/>
+      <c r="G800" s="2"/>
     </row>
     <row r="801" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G801" s="3"/>
+      <c r="G801" s="2"/>
     </row>
     <row r="802" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G802" s="3"/>
+      <c r="G802" s="2"/>
     </row>
     <row r="803" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G803" s="3"/>
+      <c r="G803" s="2"/>
     </row>
     <row r="804" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G804" s="3"/>
+      <c r="G804" s="2"/>
     </row>
     <row r="805" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G805" s="3"/>
+      <c r="G805" s="2"/>
     </row>
     <row r="806" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G806" s="3"/>
+      <c r="G806" s="2"/>
     </row>
     <row r="807" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G807" s="3"/>
+      <c r="G807" s="2"/>
     </row>
     <row r="808" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G808" s="3"/>
+      <c r="G808" s="2"/>
     </row>
     <row r="809" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G809" s="3"/>
+      <c r="G809" s="2"/>
     </row>
     <row r="810" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G810" s="3"/>
+      <c r="G810" s="2"/>
     </row>
     <row r="811" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G811" s="3"/>
+      <c r="G811" s="2"/>
     </row>
     <row r="812" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G812" s="3"/>
+      <c r="G812" s="2"/>
     </row>
     <row r="813" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G813" s="3"/>
+      <c r="G813" s="2"/>
     </row>
     <row r="814" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G814" s="3"/>
+      <c r="G814" s="2"/>
     </row>
     <row r="815" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G815" s="3"/>
+      <c r="G815" s="2"/>
     </row>
     <row r="816" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G816" s="3"/>
+      <c r="G816" s="2"/>
     </row>
     <row r="817" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G817" s="3"/>
+      <c r="G817" s="2"/>
     </row>
     <row r="818" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G818" s="3"/>
+      <c r="G818" s="2"/>
     </row>
     <row r="819" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G819" s="3"/>
+      <c r="G819" s="2"/>
     </row>
     <row r="820" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G820" s="3"/>
+      <c r="G820" s="2"/>
     </row>
     <row r="821" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G821" s="3"/>
+      <c r="G821" s="2"/>
     </row>
     <row r="822" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G822" s="3"/>
+      <c r="G822" s="2"/>
     </row>
     <row r="823" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G823" s="3"/>
+      <c r="G823" s="2"/>
     </row>
     <row r="824" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G824" s="3"/>
+      <c r="G824" s="2"/>
     </row>
     <row r="825" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G825" s="3"/>
+      <c r="G825" s="2"/>
     </row>
     <row r="826" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G826" s="3"/>
+      <c r="G826" s="2"/>
     </row>
     <row r="827" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G827" s="3"/>
+      <c r="G827" s="2"/>
     </row>
     <row r="828" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G828" s="3"/>
+      <c r="G828" s="2"/>
     </row>
     <row r="829" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G829" s="3"/>
+      <c r="G829" s="2"/>
     </row>
     <row r="830" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G830" s="3"/>
+      <c r="G830" s="2"/>
     </row>
     <row r="831" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G831" s="3"/>
+      <c r="G831" s="2"/>
     </row>
     <row r="832" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G832" s="3"/>
+      <c r="G832" s="2"/>
     </row>
     <row r="833" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G833" s="3"/>
+      <c r="G833" s="2"/>
     </row>
     <row r="834" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G834" s="3"/>
+      <c r="G834" s="2"/>
     </row>
     <row r="835" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G835" s="3"/>
+      <c r="G835" s="2"/>
     </row>
     <row r="836" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G836" s="3"/>
+      <c r="G836" s="2"/>
     </row>
     <row r="837" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G837" s="3"/>
+      <c r="G837" s="2"/>
     </row>
     <row r="838" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G838" s="3"/>
+      <c r="G838" s="2"/>
     </row>
     <row r="839" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G839" s="3"/>
+      <c r="G839" s="2"/>
     </row>
     <row r="840" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G840" s="3"/>
+      <c r="G840" s="2"/>
     </row>
     <row r="841" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G841" s="3"/>
+      <c r="G841" s="2"/>
     </row>
     <row r="842" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G842" s="3"/>
+      <c r="G842" s="2"/>
     </row>
     <row r="843" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G843" s="3"/>
+      <c r="G843" s="2"/>
     </row>
     <row r="844" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G844" s="3"/>
+      <c r="G844" s="2"/>
     </row>
     <row r="845" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G845" s="3"/>
+      <c r="G845" s="2"/>
     </row>
     <row r="846" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G846" s="3"/>
+      <c r="G846" s="2"/>
     </row>
     <row r="847" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G847" s="3"/>
+      <c r="G847" s="2"/>
     </row>
     <row r="848" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G848" s="3"/>
+      <c r="G848" s="2"/>
     </row>
     <row r="849" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G849" s="3"/>
+      <c r="G849" s="2"/>
     </row>
     <row r="850" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G850" s="3"/>
+      <c r="G850" s="2"/>
     </row>
     <row r="851" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G851" s="3"/>
+      <c r="G851" s="2"/>
     </row>
     <row r="852" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G852" s="3"/>
+      <c r="G852" s="2"/>
     </row>
     <row r="853" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G853" s="3"/>
+      <c r="G853" s="2"/>
     </row>
     <row r="854" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G854" s="3"/>
+      <c r="G854" s="2"/>
     </row>
     <row r="855" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G855" s="3"/>
+      <c r="G855" s="2"/>
     </row>
     <row r="856" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G856" s="3"/>
+      <c r="G856" s="2"/>
     </row>
     <row r="857" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G857" s="3"/>
+      <c r="G857" s="2"/>
     </row>
     <row r="858" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G858" s="3"/>
+      <c r="G858" s="2"/>
     </row>
     <row r="859" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G859" s="3"/>
+      <c r="G859" s="2"/>
     </row>
     <row r="860" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G860" s="3"/>
+      <c r="G860" s="2"/>
     </row>
     <row r="861" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G861" s="3"/>
+      <c r="G861" s="2"/>
     </row>
     <row r="862" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G862" s="3"/>
+      <c r="G862" s="2"/>
     </row>
     <row r="863" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G863" s="3"/>
+      <c r="G863" s="2"/>
     </row>
     <row r="864" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G864" s="3"/>
+      <c r="G864" s="2"/>
     </row>
     <row r="865" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G865" s="3"/>
+      <c r="G865" s="2"/>
     </row>
     <row r="866" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G866" s="3"/>
+      <c r="G866" s="2"/>
     </row>
     <row r="867" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G867" s="3"/>
+      <c r="G867" s="2"/>
     </row>
     <row r="868" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G868" s="3"/>
+      <c r="G868" s="2"/>
     </row>
     <row r="869" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G869" s="3"/>
+      <c r="G869" s="2"/>
     </row>
     <row r="870" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G870" s="3"/>
+      <c r="G870" s="2"/>
     </row>
     <row r="871" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G871" s="3"/>
+      <c r="G871" s="2"/>
     </row>
     <row r="872" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G872" s="3"/>
+      <c r="G872" s="2"/>
     </row>
     <row r="873" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G873" s="3"/>
+      <c r="G873" s="2"/>
     </row>
     <row r="874" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G874" s="3"/>
+      <c r="G874" s="2"/>
     </row>
     <row r="875" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G875" s="3"/>
+      <c r="G875" s="2"/>
     </row>
     <row r="876" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G876" s="3"/>
+      <c r="G876" s="2"/>
     </row>
     <row r="877" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G877" s="3"/>
+      <c r="G877" s="2"/>
     </row>
     <row r="878" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G878" s="3"/>
+      <c r="G878" s="2"/>
     </row>
     <row r="879" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G879" s="3"/>
+      <c r="G879" s="2"/>
     </row>
     <row r="880" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G880" s="3"/>
+      <c r="G880" s="2"/>
     </row>
     <row r="881" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G881" s="3"/>
+      <c r="G881" s="2"/>
     </row>
     <row r="882" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G882" s="3"/>
+      <c r="G882" s="2"/>
     </row>
     <row r="883" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G883" s="3"/>
+      <c r="G883" s="2"/>
     </row>
     <row r="884" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G884" s="3"/>
+      <c r="G884" s="2"/>
     </row>
     <row r="885" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G885" s="3"/>
+      <c r="G885" s="2"/>
     </row>
     <row r="886" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G886" s="3"/>
+      <c r="G886" s="2"/>
     </row>
     <row r="887" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G887" s="3"/>
+      <c r="G887" s="2"/>
     </row>
     <row r="888" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G888" s="3"/>
+      <c r="G888" s="2"/>
     </row>
     <row r="889" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G889" s="3"/>
+      <c r="G889" s="2"/>
     </row>
     <row r="890" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G890" s="3"/>
+      <c r="G890" s="2"/>
     </row>
     <row r="891" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G891" s="3"/>
+      <c r="G891" s="2"/>
     </row>
     <row r="892" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G892" s="3"/>
+      <c r="G892" s="2"/>
     </row>
     <row r="893" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G893" s="3"/>
+      <c r="G893" s="2"/>
     </row>
     <row r="894" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G894" s="3"/>
+      <c r="G894" s="2"/>
     </row>
     <row r="895" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G895" s="3"/>
+      <c r="G895" s="2"/>
     </row>
     <row r="896" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G896" s="3"/>
+      <c r="G896" s="2"/>
     </row>
     <row r="897" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G897" s="3"/>
+      <c r="G897" s="2"/>
     </row>
     <row r="898" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G898" s="3"/>
+      <c r="G898" s="2"/>
     </row>
     <row r="899" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G899" s="3"/>
+      <c r="G899" s="2"/>
     </row>
     <row r="900" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G900" s="3"/>
+      <c r="G900" s="2"/>
     </row>
     <row r="901" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G901" s="3"/>
+      <c r="G901" s="2"/>
     </row>
     <row r="902" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G902" s="3"/>
+      <c r="G902" s="2"/>
     </row>
     <row r="903" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G903" s="3"/>
+      <c r="G903" s="2"/>
     </row>
     <row r="904" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G904" s="3"/>
+      <c r="G904" s="2"/>
     </row>
     <row r="905" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G905" s="3"/>
+      <c r="G905" s="2"/>
     </row>
     <row r="906" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G906" s="3"/>
+      <c r="G906" s="2"/>
     </row>
     <row r="907" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G907" s="3"/>
+      <c r="G907" s="2"/>
     </row>
     <row r="908" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G908" s="3"/>
+      <c r="G908" s="2"/>
     </row>
     <row r="909" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G909" s="3"/>
+      <c r="G909" s="2"/>
     </row>
     <row r="910" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G910" s="3"/>
+      <c r="G910" s="2"/>
     </row>
     <row r="911" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G911" s="3"/>
+      <c r="G911" s="2"/>
     </row>
     <row r="912" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G912" s="3"/>
+      <c r="G912" s="2"/>
     </row>
     <row r="913" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G913" s="3"/>
+      <c r="G913" s="2"/>
     </row>
     <row r="914" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G914" s="3"/>
+      <c r="G914" s="2"/>
     </row>
     <row r="915" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G915" s="3"/>
+      <c r="G915" s="2"/>
     </row>
     <row r="916" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G916" s="3"/>
+      <c r="G916" s="2"/>
     </row>
     <row r="917" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G917" s="3"/>
+      <c r="G917" s="2"/>
     </row>
     <row r="918" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G918" s="3"/>
+      <c r="G918" s="2"/>
     </row>
     <row r="919" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G919" s="3"/>
+      <c r="G919" s="2"/>
     </row>
     <row r="920" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G920" s="3"/>
+      <c r="G920" s="2"/>
     </row>
     <row r="921" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G921" s="3"/>
+      <c r="G921" s="2"/>
     </row>
     <row r="922" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G922" s="3"/>
+      <c r="G922" s="2"/>
     </row>
     <row r="923" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G923" s="3"/>
+      <c r="G923" s="2"/>
     </row>
     <row r="924" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G924" s="3"/>
+      <c r="G924" s="2"/>
     </row>
     <row r="925" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G925" s="3"/>
+      <c r="G925" s="2"/>
     </row>
     <row r="926" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G926" s="3"/>
+      <c r="G926" s="2"/>
     </row>
     <row r="927" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G927" s="3"/>
+      <c r="G927" s="2"/>
     </row>
     <row r="928" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G928" s="3"/>
+      <c r="G928" s="2"/>
     </row>
     <row r="929" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G929" s="3"/>
+      <c r="G929" s="2"/>
     </row>
     <row r="930" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G930" s="3"/>
+      <c r="G930" s="2"/>
     </row>
     <row r="931" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G931" s="3"/>
+      <c r="G931" s="2"/>
     </row>
     <row r="932" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G932" s="3"/>
+      <c r="G932" s="2"/>
     </row>
     <row r="933" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G933" s="3"/>
+      <c r="G933" s="2"/>
     </row>
     <row r="934" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G934" s="3"/>
+      <c r="G934" s="2"/>
     </row>
     <row r="935" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G935" s="3"/>
+      <c r="G935" s="2"/>
     </row>
     <row r="936" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G936" s="3"/>
+      <c r="G936" s="2"/>
     </row>
     <row r="937" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G937" s="3"/>
+      <c r="G937" s="2"/>
     </row>
     <row r="938" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G938" s="3"/>
+      <c r="G938" s="2"/>
     </row>
     <row r="939" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G939" s="3"/>
+      <c r="G939" s="2"/>
     </row>
     <row r="940" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G940" s="3"/>
+      <c r="G940" s="2"/>
     </row>
     <row r="941" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G941" s="3"/>
+      <c r="G941" s="2"/>
     </row>
     <row r="942" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G942" s="3"/>
+      <c r="G942" s="2"/>
     </row>
     <row r="943" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G943" s="3"/>
+      <c r="G943" s="2"/>
     </row>
     <row r="944" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G944" s="3"/>
+      <c r="G944" s="2"/>
     </row>
     <row r="945" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G945" s="3"/>
+      <c r="G945" s="2"/>
     </row>
     <row r="946" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G946" s="3"/>
+      <c r="G946" s="2"/>
     </row>
     <row r="947" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G947" s="3"/>
+      <c r="G947" s="2"/>
     </row>
     <row r="948" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G948" s="3"/>
+      <c r="G948" s="2"/>
     </row>
     <row r="949" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G949" s="3"/>
+      <c r="G949" s="2"/>
     </row>
     <row r="950" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G950" s="3"/>
+      <c r="G950" s="2"/>
     </row>
     <row r="951" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G951" s="3"/>
+      <c r="G951" s="2"/>
     </row>
     <row r="952" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G952" s="3"/>
+      <c r="G952" s="2"/>
     </row>
     <row r="953" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G953" s="3"/>
+      <c r="G953" s="2"/>
     </row>
     <row r="954" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G954" s="3"/>
+      <c r="G954" s="2"/>
     </row>
     <row r="955" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G955" s="3"/>
+      <c r="G955" s="2"/>
     </row>
     <row r="956" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G956" s="3"/>
+      <c r="G956" s="2"/>
     </row>
     <row r="957" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G957" s="3"/>
+      <c r="G957" s="2"/>
     </row>
     <row r="958" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G958" s="3"/>
+      <c r="G958" s="2"/>
     </row>
     <row r="959" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G959" s="3"/>
+      <c r="G959" s="2"/>
     </row>
     <row r="960" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G960" s="3"/>
+      <c r="G960" s="2"/>
     </row>
     <row r="961" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G961" s="3"/>
+      <c r="G961" s="2"/>
     </row>
     <row r="962" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G962" s="3"/>
+      <c r="G962" s="2"/>
     </row>
     <row r="963" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G963" s="3"/>
+      <c r="G963" s="2"/>
     </row>
     <row r="964" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G964" s="3"/>
+      <c r="G964" s="2"/>
     </row>
     <row r="965" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G965" s="3"/>
+      <c r="G965" s="2"/>
     </row>
     <row r="966" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G966" s="3"/>
+      <c r="G966" s="2"/>
     </row>
     <row r="967" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G967" s="3"/>
+      <c r="G967" s="2"/>
     </row>
     <row r="968" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G968" s="3"/>
+      <c r="G968" s="2"/>
     </row>
     <row r="969" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G969" s="3"/>
+      <c r="G969" s="2"/>
     </row>
     <row r="970" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G970" s="3"/>
+      <c r="G970" s="2"/>
     </row>
     <row r="971" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G971" s="3"/>
+      <c r="G971" s="2"/>
     </row>
     <row r="972" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G972" s="3"/>
+      <c r="G972" s="2"/>
     </row>
     <row r="973" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G973" s="3"/>
+      <c r="G973" s="2"/>
     </row>
     <row r="974" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G974" s="3"/>
+      <c r="G974" s="2"/>
     </row>
     <row r="975" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G975" s="3"/>
+      <c r="G975" s="2"/>
     </row>
     <row r="976" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G976" s="3"/>
+      <c r="G976" s="2"/>
     </row>
     <row r="977" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G977" s="3"/>
+      <c r="G977" s="2"/>
     </row>
     <row r="978" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G978" s="3"/>
+      <c r="G978" s="2"/>
     </row>
     <row r="979" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G979" s="3"/>
+      <c r="G979" s="2"/>
     </row>
     <row r="980" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G980" s="3"/>
+      <c r="G980" s="2"/>
     </row>
     <row r="981" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G981" s="3"/>
+      <c r="G981" s="2"/>
     </row>
     <row r="982" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G982" s="3"/>
+      <c r="G982" s="2"/>
     </row>
     <row r="983" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G983" s="3"/>
+      <c r="G983" s="2"/>
     </row>
     <row r="984" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G984" s="3"/>
+      <c r="G984" s="2"/>
     </row>
     <row r="985" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G985" s="3"/>
+      <c r="G985" s="2"/>
     </row>
     <row r="986" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G986" s="3"/>
+      <c r="G986" s="2"/>
     </row>
     <row r="987" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G987" s="3"/>
+      <c r="G987" s="2"/>
     </row>
     <row r="988" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G988" s="3"/>
+      <c r="G988" s="2"/>
     </row>
     <row r="989" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G989" s="3"/>
+      <c r="G989" s="2"/>
     </row>
     <row r="990" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G990" s="3"/>
+      <c r="G990" s="2"/>
     </row>
     <row r="991" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G991" s="3"/>
+      <c r="G991" s="2"/>
     </row>
     <row r="992" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G992" s="3"/>
+      <c r="G992" s="2"/>
     </row>
     <row r="993" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G993" s="3"/>
+      <c r="G993" s="2"/>
     </row>
     <row r="994" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G994" s="3"/>
+      <c r="G994" s="2"/>
     </row>
     <row r="995" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G995" s="3"/>
+      <c r="G995" s="2"/>
     </row>
     <row r="996" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G996" s="3"/>
+      <c r="G996" s="2"/>
     </row>
     <row r="997" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G997" s="3"/>
+      <c r="G997" s="2"/>
     </row>
     <row r="998" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G998" s="3"/>
+      <c r="G998" s="2"/>
     </row>
     <row r="999" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G999" s="3"/>
+      <c r="G999" s="2"/>
     </row>
     <row r="1000" spans="7:7" ht="13" x14ac:dyDescent="0.15">
-      <c r="G1000" s="3"/>
+      <c r="G1000" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>